<commit_message>
Verify ElevenLabs findings against primary sources
Adds a Verification status section to capabilities.md: gate- and
architecture-driving claims checked against the raw docs, pricing page,
G-Cloud listing, DPA, DSPT register and status page. Corrects
versioning (tools/KB are versioned), the 31 Jul SIP outage duration,
codec wording, and drops the unsupported "AI leg only" recording claim.
Workbook basis notes updated to match; scores unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011CwCE3eafWMg1dJhL6rr3i
</commit_message>
<xml_diff>
--- a/discovery/AI Vendors/ElevenLabs/RFP_MoSCoW_ElevenLabs_draft.xlsx
+++ b/discovery/AI Vendors/ElevenLabs/RFP_MoSCoW_ElevenLabs_draft.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId3"/>
@@ -339,7 +339,7 @@
     <t xml:space="preserve">Integrates with the existing phone systems (multiple Mitel products supported by Maintel)</t>
   </si>
   <si>
-    <t xml:space="preserve">Config. Generic SIP trunk over TLS/SRTP, G.711/G.722 only (no Opus/G.729). Mitel not on ElevenLabs' compatibility list; interop is a live-test item.</t>
+    <t xml:space="preserve">Config. Generic SIP trunk over TLS/SRTP; trunk must offer G.711 or G.722 (no other codec listed). Mitel not on ElevenLabs' compatibility list; interop is a live-test item.</t>
   </si>
   <si>
     <t xml:space="preserve">TEL-02</t>
@@ -408,7 +408,7 @@
     <t xml:space="preserve">Recording either exists with retrievable retention or it does not, and its absence blocks the consent and audit design.</t>
   </si>
   <si>
-    <t xml:space="preserve">Under ZRM ElevenLabs stores nothing: recording reaches us only via the post_call_audio webhook, which is never retried, and its availability under ZRM is unconfirmed. Retention/retrieval becomes ours. AI leg only.</t>
+    <t xml:space="preserve">Under ZRM ElevenLabs stores nothing: recording reaches us only via the post_call_audio webhook, which is never retried, and its availability under ZRM is unconfirmed. Retention/retrieval becomes ours.</t>
   </si>
   <si>
     <t xml:space="preserve">TEL-09</t>
@@ -642,7 +642,7 @@
     <t xml:space="preserve">Journeys, prompts and knowledge editable by trained mydentist staff without vendor change requests (low-code / no-code)</t>
   </si>
   <si>
-    <t xml:space="preserve">No-code editors for workflows, procedures and KB; protected main branch. KB and tool edits are not versioned.</t>
+    <t xml:space="preserve">No-code editors for workflows, procedures and KB; protected main branch. Tools still need developers.</t>
   </si>
   <si>
     <t xml:space="preserve">JRN-06</t>
@@ -651,7 +651,7 @@
     <t xml:space="preserve">Test environment and version control for journey changes before release to live</t>
   </si>
   <si>
-    <t xml:space="preserve">Versions, branches, drafts, merge, traffic splits, env vars, tests per branch. KB/tools/privacy settings not versioned.</t>
+    <t xml:space="preserve">Versions, branches, drafts, merge, traffic splits, env vars, tests per branch. Privacy, retention and call limits are shared across versions.</t>
   </si>
   <si>
     <t xml:space="preserve">HND-01</t>
@@ -810,7 +810,7 @@
     <t xml:space="preserve">PCI DSS compliance</t>
   </si>
   <si>
-    <t xml:space="preserve">PCI DSS 4.0.1 Level 1 for ElevenLabs' own environment (Sep 2025). Does not take our flow out of scope.</t>
+    <t xml:space="preserve">PCI DSS for ElevenLabs' own environment (Insight Assurance, 11 Sep 2025, per G-Cloud). Does not take our flow out of scope.</t>
   </si>
   <si>
     <t xml:space="preserve">PAY-03</t>
@@ -951,7 +951,7 @@
     <t xml:space="preserve">Processing region is either UK or EEA or it is not, model inference included.</t>
   </si>
   <si>
-    <t xml:space="preserve">Assumed config: EU residency + ZRM + API-only keeps processing in the EU. No UK region; restricted LLM list; support/moderation exceptions. ZRM disables MCP.</t>
+    <t xml:space="preserve">Assumed config: EU residency + ZRM + API-only keeps processing in the EU. No UK region; under ZRM only Gemini, Claude and hosted Qwen LLMs; support/moderation exceptions. ZRM disables MCP.</t>
   </si>
   <si>
     <t xml:space="preserve">SEC-06</t>
@@ -1005,7 +1005,7 @@
     <t xml:space="preserve">Cyber Essentials Plus and/or ISO 27001 certified</t>
   </si>
   <si>
-    <t xml:space="preserve">ISO 27001:2022 (+27017/27018/27701/42001) and SOC 2 Type II. Cyber Essentials Plus labelled 2025: check currency.</t>
+    <t xml:space="preserve">ISO 27001 and Cyber Essentials Plus listed on G-Cloud; SOC 2 Type II per Trust Centre. Check certificates are current.</t>
   </si>
   <si>
     <t xml:space="preserve">REC-01</t>
@@ -1808,7 +1808,7 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1816,7 +1816,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1832,15 +1832,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="25" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="25" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1856,7 +1856,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>

</xml_diff>